<commit_message>
add 3Lab MS refactor lab TOI_8 and TOI_9
</commit_message>
<xml_diff>
--- a/MP/МониторингВAgile.xlsx
+++ b/MP/МониторингВAgile.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavel\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavel\PycharmProjects\7semTasks\MP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64CCA07B-5C5D-4EB4-85A7-54BC173110FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E53ABF6-4E68-4468-9D5D-441692254DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{39A904D6-7AF1-488B-A58D-188D3C1F603A}"/>
+    <workbookView xWindow="3465" yWindow="1815" windowWidth="21600" windowHeight="11835" xr2:uid="{39A904D6-7AF1-488B-A58D-188D3C1F603A}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>

</xml_diff>